<commit_message>
feat: Atualização de informações
</commit_message>
<xml_diff>
--- a/data_files/xlsx/FAQ_email_portal.xlsx
+++ b/data_files/xlsx/FAQ_email_portal.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricardobn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricardobn\projetos\academia-jedi\data_files\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="268">
   <si>
     <t xml:space="preserve">Prezado(a),
 Agradecemos por entrar em contato com o Centro de Estudos Jurídicos da Presidência. 
@@ -1457,6 +1457,18 @@
   </si>
   <si>
     <t>CPF, Imposto de Renda, e-cac,  aduana, evasão de divisas, CNPj, IPI, Simples. Receita Federal</t>
+  </si>
+  <si>
+    <t>Prezado visitante,
+Obrigada por entrar em contato com o Centro de Estudos Jurídicos da Presidência da República.
+Os textos do Portal da Legislação são disponibilizados em formato HTML por ser o formato mais acessível por qualquer browser, não exigindo do internauta alguma configuração específica de computador ou algum software. Isto é fator importante também para a atualização das páginas, com as constantes alterações nos Atos Normativos. Por este motivo indicamos que, sempre que possível, você consulte os atos diretamente de nossa página.
+Sugerimos que você busque softwares freeware que permitem a impressão da página visualizada em PDF, sendo possível, assim, armazenar o conteúdo.
+O Portal da Legislação disponibiliza toda a Legislação Federal para o cidadão. Acesse:
+http://www4.planalto.gov.br/legislacao
+No Portal da Legislação você pode fazer uma pesquisa em nossa base de dados, para buscar algum ato normativo específico por número, data ou termo. Acesse: 
+https://legislacao.planalto.gov.br/legisla/legislacao.nsf/fraWeb?OpenFrameSet&amp;Frame=frmWeb2&amp;Src=/legisla/legislacao.nsf%2FFrmConsultaWeb1%3FOpenForm%26AutoFramed
+Estamos à disposição para qualquer esclarecimento.
+Atenciosamente,</t>
   </si>
 </sst>
 </file>
@@ -1831,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" style="2" customWidth="1"/>
@@ -2912,6 +2924,11 @@
       </c>
       <c r="C98" s="2" t="s">
         <v>265</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="240" x14ac:dyDescent="0.25">
+      <c r="B99" s="1" t="s">
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -2925,18 +2942,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3084,18 +3101,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1CA7C12-E4E7-47A7-A0F0-D0899E6FDEC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{140B75AA-78FC-4787-BBB8-9459D7F29FEA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{140B75AA-78FC-4787-BBB8-9459D7F29FEA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1CA7C12-E4E7-47A7-A0F0-D0899E6FDEC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>